<commit_message>
First update My first git push
</commit_message>
<xml_diff>
--- a/result.xlsx
+++ b/result.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bastolaa\Box\Github\Thermodynamic-calculation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\basto\Box\Github\Thermodynamic-calculation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AA428ED-69F0-4218-A40D-6360A2C8D61E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C59345C-B9CC-462B-9F98-AB5DC08F6CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{BF8FA097-CCDC-4E0E-BE61-8D1BD0450C5D}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{BF8FA097-CCDC-4E0E-BE61-8D1BD0450C5D}"/>
   </bookViews>
   <sheets>
     <sheet name="icp" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="15">
   <si>
     <t>Al</t>
   </si>
@@ -80,21 +80,6 @@
   </si>
   <si>
     <t>type3</t>
-  </si>
-  <si>
-    <t>type4</t>
-  </si>
-  <si>
-    <t>type5</t>
-  </si>
-  <si>
-    <t>type6</t>
-  </si>
-  <si>
-    <t>type7</t>
-  </si>
-  <si>
-    <t>type8</t>
   </si>
 </sst>
 </file>
@@ -1005,7 +990,7 @@
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B21" s="2">
         <v>1.85322E-4</v>
@@ -1031,7 +1016,7 @@
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B22" s="2">
         <v>1.85322E-4</v>
@@ -1057,7 +1042,7 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B23" s="2">
         <v>1.85322E-4</v>
@@ -1083,7 +1068,7 @@
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B24" s="2">
         <v>1.85322E-4</v>
@@ -1109,7 +1094,7 @@
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="B25" s="2">
         <v>1.85322E-4</v>

</xml_diff>